<commit_message>
docs(hw2): resync anatomy.md and worksheet with the latest inspect run
anatomy.md had regressed to a run where the hand-written "## 7." defect
write-up was lost and section headers lost their numbering/spacing.
Restore the generated sections from the actual last measurement and
re-attach the defect write-up; update the worksheet's memory numbers to
match.
</commit_message>
<xml_diff>
--- a/docs/anatomy-worksheet.xlsx
+++ b/docs/anatomy-worksheet.xlsx
@@ -1,20 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" tabRatio="600" firstSheet="0" activeTab="4" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Как пользоваться" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Параметры" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="LoRA" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Память" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Ответы" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Как пользоваться" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Параметры" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LoRA" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Память" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ответы" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -25,7 +24,7 @@
     <numFmt numFmtId="165" formatCode="#,##0.0"/>
     <numFmt numFmtId="166" formatCode="0.0"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -36,30 +35,36 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="006B21A8"/>
+      <color rgb="FF6B21A8"/>
       <sz val="14"/>
     </font>
     <font>
       <name val="Calibri"/>
-      <color rgb="001A1A2E"/>
+      <color rgb="FF1A1A2E"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="001A1A2E"/>
+      <color rgb="FF1A1A2E"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
       <i val="1"/>
-      <color rgb="008888AA"/>
+      <color rgb="FF8888AA"/>
       <sz val="9"/>
     </font>
     <font>
       <name val="Consolas"/>
-      <color rgb="001A1A2E"/>
+      <color rgb="FF1A1A2E"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color rgb="FF1A1A2E"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="5">
@@ -71,17 +76,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E9D5FF"/>
+        <fgColor rgb="FFE9D5FF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF9E6"/>
+        <fgColor rgb="FFFFF9E6"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F5F0FF"/>
+        <fgColor rgb="FFF5F0FF"/>
       </patternFill>
     </fill>
   </fills>
@@ -95,21 +100,35 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00D8B4FE"/>
+        <color rgb="FFD8B4FE"/>
       </left>
       <right style="thin">
-        <color rgb="00D8B4FE"/>
+        <color rgb="FFD8B4FE"/>
       </right>
       <top style="thin">
-        <color rgb="00D8B4FE"/>
+        <color rgb="FFD8B4FE"/>
       </top>
       <bottom style="thin">
-        <color rgb="00D8B4FE"/>
+        <color rgb="FFD8B4FE"/>
       </bottom>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color rgb="00D8B4FE"/>
+        <color rgb="FFD8B4FE"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD8B4FE"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFD8B4FE"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD8B4FE"/>
       </left>
       <right/>
       <top/>
@@ -118,26 +137,13 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00D8B4FE"/>
+        <color rgb="FFD8B4FE"/>
       </left>
       <right style="thin">
-        <color rgb="00D8B4FE"/>
+        <color rgb="FFD8B4FE"/>
       </right>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="00D8B4FE"/>
-      </left>
-      <right style="thin">
-        <color rgb="00D8B4FE"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color rgb="00D8B4FE"/>
-      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -149,7 +155,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -168,32 +173,75 @@
     <xf numFmtId="165" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="2" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="8">
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="00FEE2E2"/>
+          <fgColor rgb="FFDCFCE7"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="00DCFCE7"/>
+          <fgColor rgb="FFFEE2E2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFDCFCE7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFEE2E2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFDCFCE7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFEE2E2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFDCFCE7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFEE2E2"/>
         </patternFill>
       </fill>
     </dxf>
@@ -560,21 +608,21 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="B2:B19"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
     <col width="108" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="2">
-      <c r="B2" s="4" t="inlineStr">
+    <row r="2" ht="19" customHeight="1">
+      <c r="B2" s="1" t="inlineStr">
         <is>
           <t>Сводная таблица к ДЗ 2 «Анатомия модели»</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="B3" s="2" t="inlineStr"/>
+      <c r="B3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="B4" s="2" t="inlineStr">
@@ -591,7 +639,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="2" t="inlineStr"/>
+      <c r="B6" s="2" t="n"/>
     </row>
     <row r="7">
       <c r="B7" s="3" t="inlineStr">
@@ -622,7 +670,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="2" t="inlineStr"/>
+      <c r="B11" s="2" t="n"/>
     </row>
     <row r="12">
       <c r="B12" s="3" t="inlineStr">
@@ -660,7 +708,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="2" t="inlineStr"/>
+      <c r="B17" s="2" t="n"/>
     </row>
     <row r="18">
       <c r="B18" s="3" t="inlineStr">
@@ -688,7 +736,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I18"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
@@ -701,437 +749,437 @@
     <col width="34" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+    <row r="1" ht="19" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Параметры по модулям</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>Столбцы «строк» и «столбцов» — размеры одной матрицы. «Штук» — сколько таких модулей во всей модели.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>модуль</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>штук</t>
         </is>
       </c>
-      <c r="C4" s="6" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>строк</t>
         </is>
       </c>
-      <c r="D4" s="6" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>столбцов</t>
         </is>
       </c>
-      <c r="E4" s="6" t="inlineStr">
+      <c r="E4" s="5" t="inlineStr">
         <is>
           <t>по формуле
 штук × строк × столбцов</t>
         </is>
       </c>
-      <c r="F4" s="6" t="inlineStr">
+      <c r="F4" s="5" t="inlineStr">
         <is>
           <t>по sum(p.numel())</t>
         </is>
       </c>
-      <c r="G4" s="6" t="inlineStr">
+      <c r="G4" s="5" t="inlineStr">
         <is>
           <t>сходится?</t>
         </is>
       </c>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>доля модели</t>
         </is>
       </c>
-      <c r="I4" s="6" t="inlineStr">
+      <c r="I4" s="5" t="inlineStr">
         <is>
           <t>примечание</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t>embed</t>
         </is>
       </c>
-      <c r="B5" s="8" t="n">
+      <c r="B5" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="C5" s="8" t="n">
+      <c r="C5" s="7" t="n">
         <v>151936</v>
       </c>
-      <c r="D5" s="8" t="n">
+      <c r="D5" s="7" t="n">
         <v>1024</v>
       </c>
-      <c r="E5" s="9">
+      <c r="E5" s="8">
         <f>IF(COUNT(B5:D5)=3,B5*C5*D5,"")</f>
         <v/>
       </c>
-      <c r="F5" s="10" t="n">
+      <c r="F5" s="9" t="n">
         <v>155582464</v>
       </c>
-      <c r="G5" s="11">
+      <c r="G5" s="10">
         <f>IF(E5="","—",IF(E5=F5,"сходится","РАСХОЖДЕНИЕ"))</f>
         <v/>
       </c>
-      <c r="H5" s="12">
+      <c r="H5" s="11">
         <f>IF($F$15=0,"",F5/$F$15)</f>
         <v/>
       </c>
-      <c r="I5" s="13" t="inlineStr"/>
+      <c r="I5" s="12" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>q_proj</t>
         </is>
       </c>
-      <c r="B6" s="8" t="n">
+      <c r="B6" s="7" t="n">
         <v>28</v>
       </c>
-      <c r="C6" s="8" t="n">
+      <c r="C6" s="7" t="n">
         <v>2048</v>
       </c>
-      <c r="D6" s="8" t="n">
+      <c r="D6" s="7" t="n">
         <v>1024</v>
       </c>
-      <c r="E6" s="9">
+      <c r="E6" s="8">
         <f>IF(COUNT(B6:D6)=3,B6*C6*D6,"")</f>
         <v/>
       </c>
-      <c r="F6" s="10" t="n">
+      <c r="F6" s="9" t="n">
         <v>58720256</v>
       </c>
-      <c r="G6" s="11">
+      <c r="G6" s="10">
         <f>IF(E6="","—",IF(E6=F6,"сходится","РАСХОЖДЕНИЕ"))</f>
         <v/>
       </c>
-      <c r="H6" s="12">
+      <c r="H6" s="11">
         <f>IF($F$15=0,"",F6/$F$15)</f>
         <v/>
       </c>
-      <c r="I6" s="13" t="inlineStr"/>
+      <c r="I6" s="12" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>k_proj</t>
         </is>
       </c>
-      <c r="B7" s="8" t="n">
+      <c r="B7" s="7" t="n">
         <v>28</v>
       </c>
-      <c r="C7" s="8" t="n">
+      <c r="C7" s="7" t="n">
         <v>1024</v>
       </c>
-      <c r="D7" s="8" t="n">
+      <c r="D7" s="7" t="n">
         <v>1024</v>
       </c>
-      <c r="E7" s="9">
+      <c r="E7" s="8">
         <f>IF(COUNT(B7:D7)=3,B7*C7*D7,"")</f>
         <v/>
       </c>
-      <c r="F7" s="10" t="n">
+      <c r="F7" s="9" t="n">
         <v>29360128</v>
       </c>
-      <c r="G7" s="11">
+      <c r="G7" s="10">
         <f>IF(E7="","—",IF(E7=F7,"сходится","РАСХОЖДЕНИЕ"))</f>
         <v/>
       </c>
-      <c r="H7" s="12">
+      <c r="H7" s="11">
         <f>IF($F$15=0,"",F7/$F$15)</f>
         <v/>
       </c>
-      <c r="I7" s="13" t="inlineStr"/>
+      <c r="I7" s="12" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>v_proj</t>
         </is>
       </c>
-      <c r="B8" s="8" t="n">
+      <c r="B8" s="7" t="n">
         <v>28</v>
       </c>
-      <c r="C8" s="8" t="n">
+      <c r="C8" s="7" t="n">
         <v>1024</v>
       </c>
-      <c r="D8" s="8" t="n">
+      <c r="D8" s="7" t="n">
         <v>1024</v>
       </c>
-      <c r="E8" s="9">
+      <c r="E8" s="8">
         <f>IF(COUNT(B8:D8)=3,B8*C8*D8,"")</f>
         <v/>
       </c>
-      <c r="F8" s="10" t="n">
+      <c r="F8" s="9" t="n">
         <v>29360128</v>
       </c>
-      <c r="G8" s="11">
+      <c r="G8" s="10">
         <f>IF(E8="","—",IF(E8=F8,"сходится","РАСХОЖДЕНИЕ"))</f>
         <v/>
       </c>
-      <c r="H8" s="12">
+      <c r="H8" s="11">
         <f>IF($F$15=0,"",F8/$F$15)</f>
         <v/>
       </c>
-      <c r="I8" s="13" t="inlineStr"/>
+      <c r="I8" s="12" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>o_proj</t>
         </is>
       </c>
-      <c r="B9" s="8" t="n">
+      <c r="B9" s="7" t="n">
         <v>28</v>
       </c>
-      <c r="C9" s="8" t="n">
+      <c r="C9" s="7" t="n">
         <v>1024</v>
       </c>
-      <c r="D9" s="8" t="n">
+      <c r="D9" s="7" t="n">
         <v>2048</v>
       </c>
-      <c r="E9" s="9">
+      <c r="E9" s="8">
         <f>IF(COUNT(B9:D9)=3,B9*C9*D9,"")</f>
         <v/>
       </c>
-      <c r="F9" s="10" t="n">
+      <c r="F9" s="9" t="n">
         <v>58720256</v>
       </c>
-      <c r="G9" s="11">
+      <c r="G9" s="10">
         <f>IF(E9="","—",IF(E9=F9,"сходится","РАСХОЖДЕНИЕ"))</f>
         <v/>
       </c>
-      <c r="H9" s="12">
+      <c r="H9" s="11">
         <f>IF($F$15=0,"",F9/$F$15)</f>
         <v/>
       </c>
-      <c r="I9" s="13" t="inlineStr"/>
+      <c r="I9" s="12" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="inlineStr">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>gate_proj</t>
         </is>
       </c>
-      <c r="B10" s="8" t="n">
+      <c r="B10" s="7" t="n">
         <v>28</v>
       </c>
-      <c r="C10" s="8" t="n">
+      <c r="C10" s="7" t="n">
         <v>3072</v>
       </c>
-      <c r="D10" s="8" t="n">
+      <c r="D10" s="7" t="n">
         <v>1024</v>
       </c>
-      <c r="E10" s="9">
+      <c r="E10" s="8">
         <f>IF(COUNT(B10:D10)=3,B10*C10*D10,"")</f>
         <v/>
       </c>
-      <c r="F10" s="10" t="n">
+      <c r="F10" s="9" t="n">
         <v>88080384</v>
       </c>
-      <c r="G10" s="11">
+      <c r="G10" s="10">
         <f>IF(E10="","—",IF(E10=F10,"сходится","РАСХОЖДЕНИЕ"))</f>
         <v/>
       </c>
-      <c r="H10" s="12">
+      <c r="H10" s="11">
         <f>IF($F$15=0,"",F10/$F$15)</f>
         <v/>
       </c>
-      <c r="I10" s="13" t="inlineStr"/>
+      <c r="I10" s="12" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t>up_proj</t>
         </is>
       </c>
-      <c r="B11" s="8" t="n">
+      <c r="B11" s="7" t="n">
         <v>28</v>
       </c>
-      <c r="C11" s="8" t="n">
+      <c r="C11" s="7" t="n">
         <v>3072</v>
       </c>
-      <c r="D11" s="8" t="n">
+      <c r="D11" s="7" t="n">
         <v>1024</v>
       </c>
-      <c r="E11" s="9">
+      <c r="E11" s="8">
         <f>IF(COUNT(B11:D11)=3,B11*C11*D11,"")</f>
         <v/>
       </c>
-      <c r="F11" s="10" t="n">
+      <c r="F11" s="9" t="n">
         <v>88080384</v>
       </c>
-      <c r="G11" s="11">
+      <c r="G11" s="10">
         <f>IF(E11="","—",IF(E11=F11,"сходится","РАСХОЖДЕНИЕ"))</f>
         <v/>
       </c>
-      <c r="H11" s="12">
+      <c r="H11" s="11">
         <f>IF($F$15=0,"",F11/$F$15)</f>
         <v/>
       </c>
-      <c r="I11" s="13" t="inlineStr"/>
+      <c r="I11" s="12" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="inlineStr">
+      <c r="A12" s="6" t="inlineStr">
         <is>
           <t>down_proj</t>
         </is>
       </c>
-      <c r="B12" s="8" t="n">
+      <c r="B12" s="7" t="n">
         <v>28</v>
       </c>
-      <c r="C12" s="8" t="n">
+      <c r="C12" s="7" t="n">
         <v>1024</v>
       </c>
-      <c r="D12" s="8" t="n">
+      <c r="D12" s="7" t="n">
         <v>3072</v>
       </c>
-      <c r="E12" s="9">
+      <c r="E12" s="8">
         <f>IF(COUNT(B12:D12)=3,B12*C12*D12,"")</f>
         <v/>
       </c>
-      <c r="F12" s="10" t="n">
+      <c r="F12" s="9" t="n">
         <v>88080384</v>
       </c>
-      <c r="G12" s="11">
+      <c r="G12" s="10">
         <f>IF(E12="","—",IF(E12=F12,"сходится","РАСХОЖДЕНИЕ"))</f>
         <v/>
       </c>
-      <c r="H12" s="12">
+      <c r="H12" s="11">
         <f>IF($F$15=0,"",F12/$F$15)</f>
         <v/>
       </c>
-      <c r="I12" s="13" t="inlineStr"/>
+      <c r="I12" s="12" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="inlineStr">
+      <c r="A13" s="6" t="inlineStr">
         <is>
           <t>norm</t>
         </is>
       </c>
-      <c r="B13" s="8" t="n">
+      <c r="B13" s="7" t="n">
         <v>113</v>
       </c>
-      <c r="C13" s="8" t="n"/>
-      <c r="D13" s="8" t="n"/>
-      <c r="E13" s="9">
+      <c r="C13" s="7" t="n"/>
+      <c r="D13" s="7" t="n"/>
+      <c r="E13" s="8">
         <f>IF(COUNT(B13:D13)=3,B13*C13*D13,"")</f>
         <v/>
       </c>
-      <c r="F13" s="10" t="n">
+      <c r="F13" s="9" t="n">
         <v>65536</v>
       </c>
-      <c r="G13" s="11">
+      <c r="G13" s="10">
         <f>IF(E13="","—",IF(E13=F13,"сходится","РАСХОЖДЕНИЕ"))</f>
         <v/>
       </c>
-      <c r="H13" s="12">
+      <c r="H13" s="11">
         <f>IF($F$15=0,"",F13/$F$15)</f>
         <v/>
       </c>
-      <c r="I13" s="13" t="inlineStr">
+      <c r="I13" s="12" t="inlineStr">
         <is>
           <t>вектор, а не матрица: столбцов нет</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="inlineStr">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t>lm_head</t>
         </is>
       </c>
-      <c r="B14" s="8" t="n"/>
-      <c r="C14" s="8" t="n"/>
-      <c r="D14" s="8" t="n"/>
-      <c r="E14" s="9">
+      <c r="B14" s="7" t="n"/>
+      <c r="C14" s="7" t="n"/>
+      <c r="D14" s="7" t="n"/>
+      <c r="E14" s="8">
         <f>IF(COUNT(B14:D14)=3,B14*C14*D14,"")</f>
         <v/>
       </c>
-      <c r="F14" s="10" t="n">
+      <c r="F14" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="G14" s="11">
+      <c r="G14" s="10">
         <f>IF(E14="","—",IF(E14=F14,"сходится","РАСХОЖДЕНИЕ"))</f>
         <v/>
       </c>
-      <c r="H14" s="12">
+      <c r="H14" s="11">
         <f>IF($F$15=0,"",F14/$F$15)</f>
         <v/>
       </c>
-      <c r="I14" s="13" t="inlineStr">
+      <c r="I14" s="12" t="inlineStr">
         <is>
           <t>tie_word_embeddings — своих весов нет</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="14" t="inlineStr">
+      <c r="A15" s="22" t="inlineStr">
         <is>
           <t>ИТОГО</t>
         </is>
       </c>
-      <c r="F15" s="15">
+      <c r="F15" s="14">
         <f>SUM(F5:F14)</f>
         <v/>
       </c>
-      <c r="H15" s="12">
+      <c r="H15" s="11">
         <f>IF(F15=0,"",F15/F15)</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="14" t="inlineStr">
+      <c r="A17" s="22" t="inlineStr">
         <is>
           <t>params_total из отчёта</t>
         </is>
       </c>
-      <c r="F17" s="10" t="n">
+      <c r="F17" s="9" t="n">
         <v>596049920</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="14" t="inlineStr">
+      <c r="A18" s="22" t="inlineStr">
         <is>
           <t>сумма сошлась?</t>
         </is>
       </c>
-      <c r="F18" s="11">
+      <c r="F18" s="10">
         <f>IF(F17="","заполните",IF(F15=F17,"да, сходится","НЕ СХОДИТСЯ"))</f>
         <v/>
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="F18">
+    <cfRule type="expression" priority="2" dxfId="1">
+      <formula>EXACT(F18,"НЕ СХОДИТСЯ")</formula>
+    </cfRule>
+    <cfRule type="expression" priority="4" dxfId="0">
+      <formula>EXACT(F18,"да, сходится")</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="G5:G14">
-    <cfRule type="expression" priority="1" dxfId="0">
+    <cfRule type="expression" priority="1" dxfId="1">
       <formula>EXACT(G5,"РАСХОЖДЕНИЕ")</formula>
     </cfRule>
-    <cfRule type="expression" priority="3" dxfId="1">
+    <cfRule type="expression" priority="3" dxfId="0">
       <formula>EXACT(G5,"сходится")</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F18">
-    <cfRule type="expression" priority="2" dxfId="0">
-      <formula>EXACT(F18,"НЕ СХОДИТСЯ")</formula>
-    </cfRule>
-    <cfRule type="expression" priority="4" dxfId="1">
-      <formula>EXACT(F18,"да, сходится")</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1145,317 +1193,315 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F20"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="2" max="4"/>
     <col width="26" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+    <row r="1" ht="19" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Параметры LoRA: своя формула против peft</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>На каждый целевой модуль адаптер добавляет r × (вход + выход) чисел. Умножаем на число слоёв.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="14" t="inlineStr">
+      <c r="A4" s="22" t="inlineStr">
         <is>
           <t>r (ранг)</t>
         </is>
       </c>
-      <c r="B4" s="8" t="n">
+      <c r="B4" s="7" t="n">
         <v>8</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="14" t="inlineStr">
+      <c r="A5" s="22" t="inlineStr">
         <is>
           <t>lora_alpha</t>
         </is>
       </c>
-      <c r="B5" s="8" t="n">
+      <c r="B5" s="7" t="n">
         <v>16</v>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>целевой модуль</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>слоёв</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="C7" s="5" t="inlineStr">
         <is>
           <t>вход</t>
         </is>
       </c>
-      <c r="D7" s="6" t="inlineStr">
+      <c r="D7" s="5" t="inlineStr">
         <is>
           <t>выход</t>
         </is>
       </c>
-      <c r="E7" s="6" t="inlineStr">
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>параметров адаптера
 r × (вход + выход) × слоёв</t>
         </is>
       </c>
-      <c r="F7" s="6" t="inlineStr">
+      <c r="F7" s="5" t="inlineStr">
         <is>
           <t>включён?</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>q_proj</t>
         </is>
       </c>
-      <c r="B8" s="8" t="n">
+      <c r="B8" s="7" t="n">
         <v>28</v>
       </c>
-      <c r="C8" s="8" t="n">
+      <c r="C8" s="7" t="n">
         <v>1024</v>
       </c>
-      <c r="D8" s="8" t="n">
+      <c r="D8" s="7" t="n">
         <v>2048</v>
       </c>
-      <c r="E8" s="9">
+      <c r="E8" s="8">
         <f>IF(OR(F8&lt;&gt;"да",COUNT(B8:D8)&lt;3),0,$B$4*(C8+D8)*B8)</f>
         <v/>
       </c>
-      <c r="F8" s="8" t="inlineStr">
+      <c r="F8" s="7" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>k_proj</t>
         </is>
       </c>
-      <c r="B9" s="8" t="n">
+      <c r="B9" s="7" t="n">
         <v>28</v>
       </c>
-      <c r="C9" s="8" t="n">
+      <c r="C9" s="7" t="n">
         <v>1024</v>
       </c>
-      <c r="D9" s="8" t="n">
+      <c r="D9" s="7" t="n">
         <v>1024</v>
       </c>
-      <c r="E9" s="9">
+      <c r="E9" s="8">
         <f>IF(OR(F9&lt;&gt;"да",COUNT(B9:D9)&lt;3),0,$B$4*(C9+D9)*B9)</f>
         <v/>
       </c>
-      <c r="F9" s="8" t="inlineStr">
+      <c r="F9" s="7" t="inlineStr">
         <is>
           <t>нет</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="inlineStr">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>v_proj</t>
         </is>
       </c>
-      <c r="B10" s="8" t="n">
+      <c r="B10" s="7" t="n">
         <v>28</v>
       </c>
-      <c r="C10" s="8" t="n">
+      <c r="C10" s="7" t="n">
         <v>1024</v>
       </c>
-      <c r="D10" s="8" t="n">
+      <c r="D10" s="7" t="n">
         <v>1024</v>
       </c>
-      <c r="E10" s="9">
+      <c r="E10" s="8">
         <f>IF(OR(F10&lt;&gt;"да",COUNT(B10:D10)&lt;3),0,$B$4*(C10+D10)*B10)</f>
         <v/>
       </c>
-      <c r="F10" s="8" t="inlineStr">
+      <c r="F10" s="7" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t>o_proj</t>
         </is>
       </c>
-      <c r="B11" s="8" t="n">
+      <c r="B11" s="7" t="n">
         <v>28</v>
       </c>
-      <c r="C11" s="8" t="n">
+      <c r="C11" s="7" t="n">
         <v>2048</v>
       </c>
-      <c r="D11" s="8" t="n">
+      <c r="D11" s="7" t="n">
         <v>1024</v>
       </c>
-      <c r="E11" s="9">
+      <c r="E11" s="8">
         <f>IF(OR(F11&lt;&gt;"да",COUNT(B11:D11)&lt;3),0,$B$4*(C11+D11)*B11)</f>
         <v/>
       </c>
-      <c r="F11" s="8" t="inlineStr">
+      <c r="F11" s="7" t="inlineStr">
         <is>
           <t>нет</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="inlineStr">
+      <c r="A12" s="6" t="inlineStr">
         <is>
           <t>gate_proj</t>
         </is>
       </c>
-      <c r="B12" s="8" t="n">
+      <c r="B12" s="7" t="n">
         <v>28</v>
       </c>
-      <c r="C12" s="8" t="n">
+      <c r="C12" s="7" t="n">
         <v>1024</v>
       </c>
-      <c r="D12" s="8" t="n">
+      <c r="D12" s="7" t="n">
         <v>3072</v>
       </c>
-      <c r="E12" s="9">
+      <c r="E12" s="8">
         <f>IF(OR(F12&lt;&gt;"да",COUNT(B12:D12)&lt;3),0,$B$4*(C12+D12)*B12)</f>
         <v/>
       </c>
-      <c r="F12" s="8" t="inlineStr">
+      <c r="F12" s="7" t="inlineStr">
         <is>
           <t>нет</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="inlineStr">
+      <c r="A13" s="6" t="inlineStr">
         <is>
           <t>up_proj</t>
         </is>
       </c>
-      <c r="B13" s="8" t="n">
+      <c r="B13" s="7" t="n">
         <v>28</v>
       </c>
-      <c r="C13" s="8" t="n">
+      <c r="C13" s="7" t="n">
         <v>1024</v>
       </c>
-      <c r="D13" s="8" t="n">
+      <c r="D13" s="7" t="n">
         <v>3072</v>
       </c>
-      <c r="E13" s="9">
+      <c r="E13" s="8">
         <f>IF(OR(F13&lt;&gt;"да",COUNT(B13:D13)&lt;3),0,$B$4*(C13+D13)*B13)</f>
         <v/>
       </c>
-      <c r="F13" s="8" t="inlineStr">
+      <c r="F13" s="7" t="inlineStr">
         <is>
           <t>нет</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="inlineStr">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t>down_proj</t>
         </is>
       </c>
-      <c r="B14" s="8" t="n">
+      <c r="B14" s="7" t="n">
         <v>28</v>
       </c>
-      <c r="C14" s="8" t="n">
+      <c r="C14" s="7" t="n">
         <v>3072</v>
       </c>
-      <c r="D14" s="8" t="n">
+      <c r="D14" s="7" t="n">
         <v>1024</v>
       </c>
-      <c r="E14" s="9">
+      <c r="E14" s="8">
         <f>IF(OR(F14&lt;&gt;"да",COUNT(B14:D14)&lt;3),0,$B$4*(C14+D14)*B14)</f>
         <v/>
       </c>
-      <c r="F14" s="8" t="inlineStr">
+      <c r="F14" s="7" t="inlineStr">
         <is>
           <t>нет</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="14" t="inlineStr">
+      <c r="A15" s="22" t="inlineStr">
         <is>
           <t>по вашей формуле</t>
         </is>
       </c>
-      <c r="E15" s="15">
+      <c r="E15" s="14">
         <f>SUM(E8:E14)</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="14" t="inlineStr">
+      <c r="A16" s="22" t="inlineStr">
         <is>
           <t>что показал peft</t>
         </is>
       </c>
-      <c r="E16" s="10" t="n">
+      <c r="E16" s="9" t="n">
         <v>1146880</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="14" t="inlineStr">
+      <c r="A17" s="22" t="inlineStr">
         <is>
           <t>совпало?</t>
         </is>
       </c>
-      <c r="E17" s="11">
+      <c r="E17" s="10">
         <f>IF(E16="","заполните",IF(E15=E16,"да, совпало","НЕ СОВПАЛО"))</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="14" t="inlineStr">
+      <c r="A19" s="22" t="inlineStr">
         <is>
           <t>параметров базовой модели</t>
         </is>
       </c>
-      <c r="E19" s="10" t="n">
+      <c r="E19" s="9" t="n">
         <v>596049920</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="14" t="inlineStr">
+      <c r="A20" s="22" t="inlineStr">
         <is>
           <t>доля обучаемых</t>
         </is>
       </c>
-      <c r="E20" s="16">
+      <c r="E20" s="15">
         <f>IF(E19="","",E15/E19)</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="E17">
-    <cfRule type="expression" priority="1" dxfId="0">
+    <cfRule type="expression" priority="1" dxfId="1">
       <formula>EXACT(E17,"НЕ СОВПАЛО")</formula>
     </cfRule>
-    <cfRule type="expression" priority="2" dxfId="1">
+    <cfRule type="expression" priority="2" dxfId="0">
       <formula>EXACT(E17,"да, совпало")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -1470,7 +1516,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E24"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
@@ -1479,243 +1525,243 @@
     <col width="20" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+    <row r="1" ht="19" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Память в трёх режимах</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>Пик памяти не может быть меньше весов модели ни в одном режиме. Если меньше — измерено не то.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>режим</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>пик, МБ</t>
         </is>
       </c>
-      <c r="C4" s="6" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>× к инференсу</t>
         </is>
       </c>
-      <c r="D4" s="6" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>секунд</t>
         </is>
       </c>
-      <c r="E4" s="6" t="inlineStr">
+      <c r="E4" s="5" t="inlineStr">
         <is>
           <t>пик больше весов?</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="17" t="inlineStr">
+      <c r="A5" s="16" t="inlineStr">
         <is>
           <t>инференс</t>
         </is>
       </c>
-      <c r="B5" s="18" t="n">
+      <c r="B5" s="17" t="n">
         <v>2221.5</v>
       </c>
-      <c r="C5" s="19">
+      <c r="C5" s="18">
         <f>IF($B$5="","",B5/$B$5)</f>
         <v/>
       </c>
-      <c r="D5" s="20" t="n">
-        <v>5.7</v>
-      </c>
-      <c r="E5" s="11">
+      <c r="D5" s="19" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="E5" s="10">
         <f>IF(OR(B5="",$B$14=""),"",IF(B5&gt;=$B$14,"да","МЕНЬШЕ ВЕСОВ"))</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="17" t="inlineStr">
+      <c r="A6" s="16" t="inlineStr">
         <is>
           <t>full fine-tune</t>
         </is>
       </c>
-      <c r="B6" s="18" t="n">
-        <v>6779.5</v>
-      </c>
-      <c r="C6" s="19">
+      <c r="B6" s="17" t="n">
+        <v>6715.5</v>
+      </c>
+      <c r="C6" s="18">
         <f>IF($B$5="","",B6/$B$5)</f>
         <v/>
       </c>
-      <c r="D6" s="20" t="n">
-        <v>14.1</v>
-      </c>
-      <c r="E6" s="11">
+      <c r="D6" s="19" t="n">
+        <v>21.3</v>
+      </c>
+      <c r="E6" s="10">
         <f>IF(OR(B6="",$B$14=""),"",IF(B6&gt;=$B$14,"да","МЕНЬШЕ ВЕСОВ"))</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="17" t="inlineStr">
+      <c r="A7" s="16" t="inlineStr">
         <is>
           <t>LoRA (r=8, q/v)</t>
         </is>
       </c>
-      <c r="B7" s="18" t="n">
+      <c r="B7" s="17" t="n">
         <v>3603.5</v>
       </c>
-      <c r="C7" s="19">
+      <c r="C7" s="18">
         <f>IF($B$5="","",B7/$B$5)</f>
         <v/>
       </c>
-      <c r="D7" s="20" t="n">
-        <v>5.5</v>
-      </c>
-      <c r="E7" s="11">
+      <c r="D7" s="19" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="E7" s="10">
         <f>IF(OR(B7="",$B$14=""),"",IF(B7&gt;=$B$14,"да","МЕНЬШЕ ВЕСОВ"))</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="14" t="inlineStr">
+      <c r="A9" s="22" t="inlineStr">
         <is>
           <t>Проверка на вменяемость</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="17" t="inlineStr">
+      <c r="A10" s="16" t="inlineStr">
         <is>
           <t>параметров в модели</t>
         </is>
       </c>
-      <c r="B10" s="10" t="n">
+      <c r="B10" s="9" t="n">
         <v>596049920</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="17" t="inlineStr">
+      <c r="A11" s="16" t="inlineStr">
         <is>
           <t>байт на число (bf16 = 2)</t>
         </is>
       </c>
-      <c r="B11" s="8" t="n">
+      <c r="B11" s="7" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="14" t="inlineStr">
+      <c r="A13" s="22" t="inlineStr">
         <is>
           <t>веса модели, МБ</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="21" t="n"/>
-      <c r="B14" s="9">
+      <c r="A14" s="23" t="n"/>
+      <c r="B14" s="8">
         <f>IF(COUNT(B10:B11)&lt;2,"",B10*B11/1048576)</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="14" t="inlineStr">
+      <c r="A16" s="22" t="inlineStr">
         <is>
           <t>Условия замера — без них числа ничего не значат</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="17" t="inlineStr">
+      <c r="A17" s="16" t="inlineStr">
         <is>
           <t>устройство (cpu / cuda / mps)</t>
         </is>
       </c>
-      <c r="B17" s="22" t="inlineStr">
+      <c r="B17" s="20" t="inlineStr">
         <is>
           <t>mps</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="17" t="inlineStr">
+      <c r="A18" s="16" t="inlineStr">
         <is>
           <t>чем меряли память</t>
         </is>
       </c>
-      <c r="B18" s="22" t="inlineStr">
+      <c r="B18" s="20" t="inlineStr">
         <is>
           <t>torch.mps.driver_allocated_memory (аллокатор mps)</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="17" t="inlineStr">
+      <c r="A19" s="16" t="inlineStr">
         <is>
           <t>dtype</t>
         </is>
       </c>
-      <c r="B19" s="22" t="inlineStr">
+      <c r="B19" s="20" t="inlineStr">
         <is>
           <t>bfloat16</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="17" t="inlineStr">
+      <c r="A20" s="16" t="inlineStr">
         <is>
           <t>seq_len</t>
         </is>
       </c>
-      <c r="B20" s="22" t="n">
+      <c r="B20" s="20" t="n">
         <v>256</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="17" t="inlineStr">
+      <c r="A21" s="16" t="inlineStr">
         <is>
           <t>batch_size</t>
         </is>
       </c>
-      <c r="B21" s="22" t="n">
+      <c r="B21" s="20" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="17" t="inlineStr">
+      <c r="A22" s="16" t="inlineStr">
         <is>
           <t>сколько раз повторяли замер</t>
         </is>
       </c>
-      <c r="B22" s="22" t="n">
+      <c r="B22" s="20" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="17" t="inlineStr">
+      <c r="A23" s="16" t="inlineStr">
         <is>
           <t>что именно в шаге (forward / +backward / +optimizer)</t>
         </is>
       </c>
-      <c r="B23" s="22" t="inlineStr">
+      <c r="B23" s="20" t="inlineStr">
         <is>
           <t>инференс — только forward; full_ft и lora — forward + backward + optimizer.step()</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="17" t="inlineStr">
+      <c r="A24" s="16" t="inlineStr">
         <is>
           <t>модель</t>
         </is>
       </c>
-      <c r="B24" s="22" t="inlineStr">
+      <c r="B24" s="20" t="inlineStr">
         <is>
           <t>Qwen/Qwen3-0.6B</t>
         </is>
@@ -1726,10 +1772,10 @@
     <mergeCell ref="A13:A14"/>
   </mergeCells>
   <conditionalFormatting sqref="E5:E7">
-    <cfRule type="expression" priority="1" dxfId="0">
+    <cfRule type="expression" priority="1" dxfId="1">
       <formula>EXACT(E5,"МЕНЬШЕ ВЕСОВ")</formula>
     </cfRule>
-    <cfRule type="expression" priority="2" dxfId="1">
+    <cfRule type="expression" priority="2" dxfId="0">
       <formula>EXACT(E5,"да")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -1744,94 +1790,114 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
     <col width="58" customWidth="1" min="2" max="2"/>
     <col width="80" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+    <row r="1" ht="19" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Почему ваши числа именно такие</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>Своими словами. Одного-двух предложений достаточно — но они должны быть про ваши числа, а не про чужие.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="6" t="inlineStr"/>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="A4" s="5" t="n"/>
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>вопрос</t>
         </is>
       </c>
-      <c r="C4" s="6" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>ваш ответ</t>
         </is>
       </c>
     </row>
     <row r="5" ht="58" customHeight="1">
-      <c r="A5" s="14" t="n">
+      <c r="A5" s="22" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="23" t="inlineStr">
+      <c r="B5" s="21" t="inlineStr">
         <is>
           <t>Почему lm_head в вашей таблице весит столько, сколько весит?</t>
         </is>
       </c>
-      <c r="C5" s="24" t="n"/>
+      <c r="C5" s="24" t="inlineStr">
+        <is>
+          <t>lm_head весит 0 параметров, потому что tie_word_embeddings=True: его вес - это тот же тензор embed_tokens.weight (151936×1024), а не отдельная матрица; в named_parameters() он встречается второй раз и помечается tied=True, поэтому в сумму не идёт.</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="58" customHeight="1">
-      <c r="A6" s="14" t="n">
+      <c r="A6" s="22" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="23" t="inlineStr">
+      <c r="B6" s="21" t="inlineStr">
         <is>
           <t>Почему k_proj вдвое меньше q_proj?</t>
         </is>
       </c>
-      <c r="C6" s="24" t="n"/>
+      <c r="C6" s="24" t="inlineStr">
+        <is>
+          <t>Это GQA: 16 голов запроса, но всего 8 KV-голов при head_dim=128. q_proj проецирует в 16×128=2048, а k_proj (как и v_proj) - только в 8×128=1024, то есть ровно вдвое меньше выходных признаков при одинаковом hidden_size=1024 на входе.</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="58" customHeight="1">
-      <c r="A7" s="14" t="n">
+      <c r="A7" s="22" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="23" t="inlineStr">
+      <c r="B7" s="21" t="inlineStr">
         <is>
           <t>Почему MLP занимает большую долю модели, чем всё внимание вместе?</t>
         </is>
       </c>
-      <c r="C7" s="24" t="n"/>
+      <c r="C7" s="24" t="inlineStr">
+        <is>
+          <t>На каждый блок MLP - три матрицы (gate/up/down) размера 3072×1024, суммарно 264 241 152 параметров, а внимание — четыре матрицы (q/k/v/o) суммарно 176 160 768: 44.3% модели против 29.5%. intermediate_size (3072) втрое больше hidden_size (1024), а проекций в MLP на одну больше, чем эффективных в attention из-за GQA.</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="58" customHeight="1">
-      <c r="A8" s="14" t="n">
+      <c r="A8" s="22" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="23" t="inlineStr">
+      <c r="B8" s="21" t="inlineStr">
         <is>
           <t>Почему при 0,192% обучаемых параметров LoRA экономит намного больше памяти, чем 0,192%?</t>
         </is>
       </c>
-      <c r="C8" s="24" t="n"/>
+      <c r="C8" s="24" t="inlineStr">
+        <is>
+          <t>0.192% - это доля обучаемых параметров, а память экономится не на них одних: full fine-tune хранит градиенты и два состояния AdamW для ВСЕХ 596M весов (≈×4 к весам ещё до активаций), тогда как LoRA считает градиенты и optimizer state только для 1 146 880 параметров адаптера. Экономится в основном самая тяжёлая часть — градиенты/оптимизатор базовой модели, а не активации, которые в обоих режимах сопоставимы.</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="58" customHeight="1">
-      <c r="A9" s="14" t="n">
+      <c r="A9" s="22" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="23" t="inlineStr">
+      <c r="B9" s="21" t="inlineStr">
         <is>
           <t>Ваша метрика памяти — какая и почему именно она подходит вашему устройству?</t>
         </is>
       </c>
-      <c r="C9" s="24" t="n"/>
+      <c r="C9" s="24" t="inlineStr">
+        <is>
+          <t>torch.mps.driver_allocated_memory - показания аллокатора Metal/MPS. На устройстве mps тензоры лежат не в host RSS процесса (ru_maxrss её почти не видит, см. Дефект 4 в anatomy.md), а в памяти, которой управляет MPS-драйвер, поэтому только его собственный счётчик отражает реальный расход весов/градиентов/активаций на этом устройстве.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>